<commit_message>
workflow -> scenario add hrex requirements move error groups into the PAS Scenarios group additional refactors around must support client tests
</commit_message>
<xml_diff>
--- a/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
+++ b/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-pas-test-kit/lib/davinci_pas_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8115E68B-45AF-3F43-9D3B-81B26D0AE85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ECB3255-5701-D742-A5D1-E246EC744CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="453">
   <si>
     <r>
       <rPr>
@@ -2733,6 +2733,24 @@
   </si>
   <si>
     <t>Updated actor - Client is responsible for the Claim</t>
+  </si>
+  <si>
+    <t>Data Sources **SHALL** be capable of populating the data element when sharing resources compliant with the profile.</t>
+  </si>
+  <si>
+    <t>hrex-conf-1</t>
+  </si>
+  <si>
+    <t>https://hl7.org/fhir/us/davinci-hrex/1.2.0/en/conformance.html#ci-c-conf-1</t>
+  </si>
+  <si>
+    <t>hrex-conf-2</t>
+  </si>
+  <si>
+    <t>Data Consumers **SHALL** be capable of processing resource instances containing the data elements without generating an error or causing the application to fail.</t>
+  </si>
+  <si>
+    <t>https://hl7.org/fhir/us/davinci-hrex/1.2.0/en/conformance.html#ci-c-conf-2</t>
   </si>
 </sst>
 </file>
@@ -6571,12 +6589,46 @@
       </c>
       <c r="R120" s="10"/>
     </row>
-    <row r="121" spans="1:21" ht="16" x14ac:dyDescent="0.2">
-      <c r="B121" s="11"/>
+    <row r="121" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+      <c r="A121" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="B121" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E121" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="G121" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="R121" s="10"/>
     </row>
-    <row r="122" spans="1:21" ht="16" x14ac:dyDescent="0.2">
-      <c r="B122" s="11"/>
+    <row r="122" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+      <c r="A122" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="B122" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="C122" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="D122" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E122" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="G122" s="7" t="b">
+        <v>0</v>
+      </c>
       <c r="R122" s="10"/>
     </row>
     <row r="123" spans="1:21" ht="16" x14ac:dyDescent="0.2">
@@ -8557,6 +8609,8 @@
     <hyperlink ref="B52" r:id="rId3" location="ci-c-spec-11" xr:uid="{4E0F9A5A-0897-2C4B-98E8-127D0E73D6C1}"/>
     <hyperlink ref="B106" r:id="rId4" location="ci-c-spec-65" xr:uid="{2C76CA9A-AF34-C946-9996-4CD6012F10C0}"/>
     <hyperlink ref="B67" r:id="rId5" location="ci-c-spec-26" xr:uid="{2791CF85-461B-1340-B643-634665A3629B}"/>
+    <hyperlink ref="B121" r:id="rId6" location="ci-c-conf-1" xr:uid="{F9502762-2CAC-054B-AC35-8FE364937A33}"/>
+    <hyperlink ref="B122" r:id="rId7" location="ci-c-conf-2" xr:uid="{B9020D2D-CDEC-9B45-9DBE-D41FF8F58455}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -8818,6 +8872,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -9071,7 +9134,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
@@ -9084,16 +9147,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12FB330C-B068-4EE3-928A-A72A297ABA91}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9113,7 +9175,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -9129,12 +9191,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>